<commit_message>
Ataulização dos resultados de Agosto fechados
</commit_message>
<xml_diff>
--- a/Indicadores_Performance_Comercial.xlsx
+++ b/Indicadores_Performance_Comercial.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17ab24b3b76d94b1/Desktop/Apresentação de Mídia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="11_73CBF7718050DB9A570585A2C493DFA2F5AB32E3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB94AB9D-8C2E-4685-B509-BB751E079A3A}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="11_73CBF7718050DB9A570585A2C493DFA2F5AB32E3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DCDC1646-2AC0-4CD9-828F-E4F452558FAA}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,6 @@
     <sheet name="Indicadores" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="33">
   <si>
     <t>Dados brutos — Agendamento, Reunião e Contrato fechado</t>
   </si>
@@ -680,7 +679,9 @@
       <c r="H5" s="6">
         <v>41</v>
       </c>
-      <c r="I5" s="6"/>
+      <c r="I5" s="6">
+        <v>57</v>
+      </c>
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
       <c r="L5" s="6"/>
@@ -711,7 +712,9 @@
       <c r="H6" s="6">
         <v>42</v>
       </c>
-      <c r="I6" s="6"/>
+      <c r="I6" s="6">
+        <v>37</v>
+      </c>
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
       <c r="L6" s="6"/>
@@ -778,7 +781,7 @@
       </c>
       <c r="I8" s="8">
         <f t="shared" ref="I8" si="2">SUM(I5:I7)</f>
-        <v>0</v>
+        <v>94</v>
       </c>
       <c r="J8" s="8">
         <f t="shared" ref="J8" si="3">SUM(J5:J7)</f>
@@ -880,7 +883,9 @@
       <c r="H12" s="6">
         <v>30</v>
       </c>
-      <c r="I12" s="6"/>
+      <c r="I12" s="6">
+        <v>37</v>
+      </c>
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
       <c r="L12" s="6"/>
@@ -911,7 +916,9 @@
       <c r="H13" s="6">
         <v>35</v>
       </c>
-      <c r="I13" s="6"/>
+      <c r="I13" s="6">
+        <v>21</v>
+      </c>
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
       <c r="L13" s="6"/>
@@ -978,7 +985,7 @@
       </c>
       <c r="I15" s="8">
         <f t="shared" ref="I15" si="9">SUM(I12:I14)</f>
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="J15" s="8">
         <f t="shared" ref="J15" si="10">SUM(J12:J14)</f>
@@ -1080,7 +1087,9 @@
       <c r="H19" s="6">
         <v>4</v>
       </c>
-      <c r="I19" s="6"/>
+      <c r="I19" s="6">
+        <v>3</v>
+      </c>
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
       <c r="L19" s="6"/>
@@ -1111,7 +1120,9 @@
       <c r="H20" s="6">
         <v>3</v>
       </c>
-      <c r="I20" s="6"/>
+      <c r="I20" s="6">
+        <v>4</v>
+      </c>
       <c r="J20" s="6"/>
       <c r="K20" s="6"/>
       <c r="L20" s="6"/>
@@ -1170,7 +1181,7 @@
       </c>
       <c r="I22" s="8">
         <f t="shared" ref="I22" si="16">SUM(I19:I21)</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J22" s="8">
         <f t="shared" ref="J22" si="17">SUM(J19:J21)</f>
@@ -1201,14 +1212,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="9" width="12" customWidth="1"/>
+    <col min="2" max="10" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16.899999999999999" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:11" ht="16.899999999999999" x14ac:dyDescent="0.5">
       <c r="A1" s="16" t="s">
         <v>15</v>
       </c>
@@ -1221,8 +1232,9 @@
       <c r="H1" s="16"/>
       <c r="I1" s="16"/>
       <c r="J1" s="16"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="K1" s="16"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="9" t="s">
         <v>16</v>
       </c>
@@ -1234,8 +1246,9 @@
       <c r="G3" s="10"/>
       <c r="H3" s="10"/>
       <c r="I3" s="10"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="J3" s="10"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1261,10 +1274,13 @@
         <v>27</v>
       </c>
       <c r="I4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="5" t="s">
         <v>9</v>
       </c>
@@ -1296,12 +1312,16 @@
         <f>IFERROR(Dados!H12/Dados!H5,"")</f>
         <v>0.73170731707317072</v>
       </c>
-      <c r="I5" s="12">
+      <c r="I5" s="11">
+        <f>IFERROR(Dados!I12/Dados!I5,"")</f>
+        <v>0.64912280701754388</v>
+      </c>
+      <c r="J5" s="12">
         <f>IFERROR(SUM(Dados!B12:G12)/SUM(Dados!B5:G5),"")</f>
         <v>0.56470588235294117</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" s="5" t="s">
         <v>10</v>
       </c>
@@ -1333,12 +1353,16 @@
         <f>IFERROR(Dados!H13/Dados!H6,"")</f>
         <v>0.83333333333333337</v>
       </c>
-      <c r="I6" s="12">
+      <c r="I6" s="11">
+        <f>IFERROR(Dados!I13/Dados!I6,"")</f>
+        <v>0.56756756756756754</v>
+      </c>
+      <c r="J6" s="12">
         <f>IFERROR(SUM(Dados!B13:G13)/SUM(Dados!B6:G6),"")</f>
         <v>0.74089068825910931</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="5" t="s">
         <v>11</v>
       </c>
@@ -1370,12 +1394,13 @@
         <f>IFERROR(Dados!H14/Dados!H7,"")</f>
         <v/>
       </c>
-      <c r="I7" s="12">
+      <c r="I7" s="11"/>
+      <c r="J7" s="12">
         <f>IFERROR(SUM(Dados!B14:G14)/SUM(Dados!B7:G7),"")</f>
         <v>0.45977011494252873</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" s="13" t="s">
         <v>18</v>
       </c>
@@ -1404,12 +1429,13 @@
         <v>0.72289156626506024</v>
       </c>
       <c r="H8" s="14"/>
-      <c r="I8" s="14">
+      <c r="I8" s="14"/>
+      <c r="J8" s="14">
         <f>IFERROR(SUM(Dados!B15:G15)/SUM(Dados!B8:G8),"")</f>
         <v>0.63293650793650791</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="9" t="s">
         <v>19</v>
       </c>
@@ -1421,8 +1447,9 @@
       <c r="G10" s="10"/>
       <c r="H10" s="10"/>
       <c r="I10" s="10"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="J10" s="10"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
         <v>2</v>
       </c>
@@ -1448,10 +1475,13 @@
         <v>27</v>
       </c>
       <c r="I11" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J11" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A12" s="5" t="s">
         <v>9</v>
       </c>
@@ -1483,12 +1513,16 @@
         <f>IFERROR(Dados!H19/Dados!H12,"")</f>
         <v>0.13333333333333333</v>
       </c>
-      <c r="I12" s="12">
+      <c r="I12" s="11">
+        <f>IFERROR(Dados!I19/Dados!I12,"")</f>
+        <v>8.1081081081081086E-2</v>
+      </c>
+      <c r="J12" s="12">
         <f>IFERROR(SUM(Dados!B19:G19)/SUM(Dados!B12:G12),"")</f>
         <v>0.19791666666666666</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A13" s="5" t="s">
         <v>10</v>
       </c>
@@ -1520,12 +1554,16 @@
         <f>IFERROR(Dados!H20/Dados!H13,"")</f>
         <v>8.5714285714285715E-2</v>
       </c>
-      <c r="I13" s="12">
+      <c r="I13" s="11">
+        <f>IFERROR(Dados!I20/Dados!I13,"")</f>
+        <v>0.19047619047619047</v>
+      </c>
+      <c r="J13" s="12">
         <f>IFERROR(SUM(Dados!B20:G20)/SUM(Dados!B13:G13),"")</f>
         <v>0.15300546448087432</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A14" s="5" t="s">
         <v>11</v>
       </c>
@@ -1557,12 +1595,13 @@
         <f>IFERROR(Dados!H21/Dados!H14,"")</f>
         <v/>
       </c>
-      <c r="I14" s="12">
+      <c r="I14" s="11"/>
+      <c r="J14" s="12">
         <f>IFERROR(SUM(Dados!B21:G21)/SUM(Dados!B14:G14),"")</f>
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A15" s="13" t="s">
         <v>18</v>
       </c>
@@ -1591,12 +1630,13 @@
         <v>8.3333333333333329E-2</v>
       </c>
       <c r="H15" s="14"/>
-      <c r="I15" s="14">
+      <c r="I15" s="14"/>
+      <c r="J15" s="14">
         <f>IFERROR(SUM(Dados!B22:G22)/SUM(Dados!B15:G15),"")</f>
         <v>0.15047021943573669</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A17" s="9" t="s">
         <v>20</v>
       </c>
@@ -1608,8 +1648,9 @@
       <c r="G17" s="10"/>
       <c r="H17" s="10"/>
       <c r="I17" s="10"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J17" s="10"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A18" s="3" t="s">
         <v>2</v>
       </c>
@@ -1635,10 +1676,13 @@
         <v>27</v>
       </c>
       <c r="I18" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J18" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A19" s="5" t="s">
         <v>9</v>
       </c>
@@ -1670,12 +1714,16 @@
         <f>IFERROR(Dados!H19/Dados!H5,"")</f>
         <v>9.7560975609756101E-2</v>
       </c>
-      <c r="I19" s="12">
+      <c r="I19" s="11">
+        <f>IFERROR(Dados!I19/Dados!I5,"")</f>
+        <v>5.2631578947368418E-2</v>
+      </c>
+      <c r="J19" s="12">
         <f>IFERROR(SUM(Dados!B19:G19)/SUM(Dados!B5:G5),"")</f>
         <v>0.11176470588235295</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A20" s="5" t="s">
         <v>10</v>
       </c>
@@ -1707,12 +1755,16 @@
         <f>IFERROR(Dados!H20/Dados!H6,"")</f>
         <v>7.1428571428571425E-2</v>
       </c>
-      <c r="I20" s="12">
+      <c r="I20" s="11">
+        <f>IFERROR(Dados!I20/Dados!I6,"")</f>
+        <v>0.10810810810810811</v>
+      </c>
+      <c r="J20" s="12">
         <f>IFERROR(SUM(Dados!B20:G20)/SUM(Dados!B6:G6),"")</f>
         <v>0.11336032388663968</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A21" s="5" t="s">
         <v>11</v>
       </c>
@@ -1744,12 +1796,13 @@
         <f>IFERROR(Dados!H21/Dados!H7,"")</f>
         <v/>
       </c>
-      <c r="I21" s="12">
+      <c r="I21" s="11"/>
+      <c r="J21" s="12">
         <f>IFERROR(SUM(Dados!B21:G21)/SUM(Dados!B7:G7),"")</f>
         <v>1.1494252873563218E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A22" s="13" t="s">
         <v>18</v>
       </c>
@@ -1778,12 +1831,13 @@
         <v>6.0240963855421686E-2</v>
       </c>
       <c r="H22" s="14"/>
-      <c r="I22" s="14">
+      <c r="I22" s="14"/>
+      <c r="J22" s="14">
         <f>IFERROR(SUM(Dados!B22:G22)/SUM(Dados!B8:G8),"")</f>
         <v>9.5238095238095233E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A25" s="9" t="s">
         <v>21</v>
       </c>
@@ -1795,8 +1849,9 @@
       <c r="G25" s="10"/>
       <c r="H25" s="10"/>
       <c r="I25" s="10"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J25" s="10"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A26" s="3" t="s">
         <v>22</v>
       </c>
@@ -1821,8 +1876,11 @@
       <c r="H26" s="4" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="I26" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A27" s="5" t="s">
         <v>23</v>
       </c>
@@ -1851,17 +1909,21 @@
         <v>6.0240963855421686E-2</v>
       </c>
       <c r="H27" s="11">
-        <f t="shared" ref="H27" si="1">H22</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.45">
+        <f t="shared" ref="H27:I27" si="1">H22</f>
+        <v>0</v>
+      </c>
+      <c r="I27" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A28" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B28" s="15"/>
       <c r="C28" s="11">
-        <f t="shared" ref="C28:H28" si="2">IFERROR((C27-B27),"")</f>
+        <f t="shared" ref="C28:I28" si="2">IFERROR((C27-B27),"")</f>
         <v>4.4383561643835612E-2</v>
       </c>
       <c r="D28" s="11">
@@ -1884,8 +1946,12 @@
         <f t="shared" si="2"/>
         <v>-6.0240963855421686E-2</v>
       </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="I28" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A29" s="5" t="s">
         <v>25</v>
       </c>
@@ -1893,7 +1959,7 @@
         <v>26</v>
       </c>
       <c r="C29" s="15" t="str">
-        <f t="shared" ref="C29:H29" si="3">IF(C28="","—",IF(C28&gt;=0,"Evolução","Involução"))</f>
+        <f t="shared" ref="C29:I29" si="3">IF(C28="","—",IF(C28&gt;=0,"Evolução","Involução"))</f>
         <v>Evolução</v>
       </c>
       <c r="D29" s="15" t="str">
@@ -1916,10 +1982,14 @@
         <f t="shared" si="3"/>
         <v>Involução</v>
       </c>
+      <c r="I29" s="15" t="str">
+        <f t="shared" si="3"/>
+        <v>Evolução</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>